<commit_message>
Six more paintings, and the placeholders they replace
The Morrigan's Avatar, The Whisperer, The Devil Kings Avatar, Archangel
Skyrehaal, Barlgowrath and Sinbad-Sinodess all had their own paintings and
were still wearing borrowed ones. The Morrigan's Avatar had the picture of
the Titan herself, which is the god she is sent in place of, so that one was
wrong rather than merely stand-in.

Eight named characters are still borrowing, and eleven still have nothing.

The filenames came back with the lineage tacked on, as "Barlgowrath -
Ancient Beast, demonic war-leader", because that is how the prompt sheet
labels them. Rather than add those exact spellings the matcher now falls back
to the name before the dash. It tries the whole name first, so the ones where
the dash is part of who they are, like Hannarial Icetear - Captain of the Red
Rangers, still match themselves.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/blood-of-icetear-cards.xlsx
+++ b/docs/blood-of-icetear-cards.xlsx
@@ -720,7 +720,7 @@
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>corrupted-angel.webp</t>
+          <t>devil-kings-avatar.webp</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>golden-angel.webp</t>
+          <t>archangel-skyrehaal.webp</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>morrigan.jpg</t>
+          <t>morrigan-avatar.webp</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>sinbad-sinodess.jpg</t>
+          <t>sinbad-sinodess.webp</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>lucifials-avatar.jpg</t>
+          <t>whisperer.webp</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>spider-horror.webp</t>
+          <t>barlgowrath.webp</t>
         </is>
       </c>
     </row>

</xml_diff>